<commit_message>
Track Yutori-sourced links separately in progress xlsx; widen /yutori window to 5d
- .claude/commands/yutori.md: newer_than 3d -> 5d, ώστε να καλύπτεται και το
  τετραήμερο κενό Πέμπτη -> Δευτέρα της υπενθύμισης. Το βήμα του xlsx πλέον
  καλεί το script αντί να προσθέτει γραμμή με το χέρι.
- scripts/build_progress_xlsx.py: διαχωρισμός συνδέσμων ανά πηγή με βάση την
  ένδειξη «(via Yutori Scout)». Νέες στήλες «Λοιπές πηγές (web)» και
  «via Yutori Scout», σωρευτικό στη στήλη E.
- Το ημερήσιο γράφημα έγινε στοιβαγμένο (web + Yutori) ώστε να φαίνεται η
  συνεισφορά κάθε πηγής· η σύνοψη ανά μήνα απέκτησε στήλη «εκ των οποίων
  via Yutori».

Τρέχουσα κατανομή: 334 links, εκ των οποίων 101 via Yutori Scout.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ΠΡΟΟΔΟΣ_ΣΥΛΛΟΓΗΣ_2026.xlsx
+++ b/ΠΡΟΟΔΟΣ_ΣΥΛΛΟΓΗΣ_2026.xlsx
@@ -186,7 +186,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Νέα links ανά ημέρα — Δασικές Πυρκαγιές Ελλάδα 2026</a:t>
+              <a:t>Νέα links ανά ημέρα ανά πηγή — Δασικές Πυρκαγιές Ελλάδα 2026</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -195,13 +195,13 @@
     <plotArea>
       <barChart>
         <barDir val="col"/>
-        <grouping val="clustered"/>
+        <grouping val="stacked"/>
         <ser>
           <idx val="0"/>
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Ημερήσια Πρόοδος'!B1</f>
+              <f>'Ημερήσια Πρόοδος'!C1</f>
             </strRef>
           </tx>
           <spPr>
@@ -216,11 +216,36 @@
           </cat>
           <val>
             <numRef>
-              <f>'Ημερήσια Πρόοδος'!$B$2:$B$108</f>
+              <f>'Ημερήσια Πρόοδος'!$C$2:$C$108</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'Ημερήσια Πρόοδος'!D1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Ημερήσια Πρόοδος'!$A$3:$A$108</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Ημερήσια Πρόοδος'!$D$2:$D$108</f>
             </numRef>
           </val>
         </ser>
         <gapWidth val="40"/>
+        <overlap val="100"/>
         <axId val="10"/>
         <axId val="100"/>
       </barChart>
@@ -281,6 +306,9 @@
         <crossAx val="10"/>
       </valAx>
     </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
     <plotVisOnly val="1"/>
     <dispBlanksAs val="gap"/>
   </chart>
@@ -313,7 +341,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Ημερήσια Πρόοδος'!C1</f>
+              <f>'Ημερήσια Πρόοδος'!E1</f>
             </strRef>
           </tx>
           <spPr>
@@ -336,7 +364,7 @@
           </cat>
           <val>
             <numRef>
-              <f>'Ημερήσια Πρόοδος'!$C$2:$C$108</f>
+              <f>'Ημερήσια Πρόοδος'!$E$2:$E$108</f>
             </numRef>
           </val>
         </ser>
@@ -410,7 +438,7 @@
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
-      <col>4</col>
+      <col>6</col>
       <colOff>0</colOff>
       <row>1</row>
       <rowOff>0</rowOff>
@@ -432,7 +460,7 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>4</col>
+      <col>6</col>
       <colOff>0</colOff>
       <row>21</row>
       <rowOff>0</rowOff>
@@ -744,12 +772,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C108"/>
+  <dimension ref="A1:E108"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -765,6 +795,16 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>Λοιπές πηγές (web)</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>via Yutori Scout</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>Σύνολο Links</t>
         </is>
       </c>
@@ -781,6 +821,12 @@
       <c r="C2" s="2" t="n">
         <v>11</v>
       </c>
+      <c r="D2" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -792,6 +838,12 @@
         <v>10</v>
       </c>
       <c r="C3" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" s="3" t="n">
         <v>21</v>
       </c>
     </row>
@@ -805,6 +857,12 @@
         <v>1</v>
       </c>
       <c r="C4" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" s="3" t="n">
         <v>22</v>
       </c>
     </row>
@@ -818,6 +876,12 @@
         <v>0</v>
       </c>
       <c r="C5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" s="3" t="n">
         <v>22</v>
       </c>
     </row>
@@ -831,6 +895,12 @@
         <v>0</v>
       </c>
       <c r="C6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" s="3" t="n">
         <v>22</v>
       </c>
     </row>
@@ -844,6 +914,12 @@
         <v>0</v>
       </c>
       <c r="C7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" s="3" t="n">
         <v>22</v>
       </c>
     </row>
@@ -857,6 +933,12 @@
         <v>0</v>
       </c>
       <c r="C8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" s="3" t="n">
         <v>22</v>
       </c>
     </row>
@@ -870,6 +952,12 @@
         <v>0</v>
       </c>
       <c r="C9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" s="3" t="n">
         <v>22</v>
       </c>
     </row>
@@ -883,6 +971,12 @@
         <v>0</v>
       </c>
       <c r="C10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" s="3" t="n">
         <v>22</v>
       </c>
     </row>
@@ -896,6 +990,12 @@
         <v>0</v>
       </c>
       <c r="C11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" s="3" t="n">
         <v>22</v>
       </c>
     </row>
@@ -909,6 +1009,12 @@
         <v>0</v>
       </c>
       <c r="C12" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D12" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" s="3" t="n">
         <v>22</v>
       </c>
     </row>
@@ -922,6 +1028,12 @@
         <v>0</v>
       </c>
       <c r="C13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" s="3" t="n">
         <v>22</v>
       </c>
     </row>
@@ -935,6 +1047,12 @@
         <v>0</v>
       </c>
       <c r="C14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" s="3" t="n">
         <v>22</v>
       </c>
     </row>
@@ -948,6 +1066,12 @@
         <v>0</v>
       </c>
       <c r="C15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" s="3" t="n">
         <v>22</v>
       </c>
     </row>
@@ -961,6 +1085,12 @@
         <v>0</v>
       </c>
       <c r="C16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" s="3" t="n">
         <v>22</v>
       </c>
     </row>
@@ -974,6 +1104,12 @@
         <v>0</v>
       </c>
       <c r="C17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" s="3" t="n">
         <v>22</v>
       </c>
     </row>
@@ -987,6 +1123,12 @@
         <v>0</v>
       </c>
       <c r="C18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E18" s="3" t="n">
         <v>22</v>
       </c>
     </row>
@@ -1000,6 +1142,12 @@
         <v>0</v>
       </c>
       <c r="C19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" s="3" t="n">
         <v>22</v>
       </c>
     </row>
@@ -1013,6 +1161,12 @@
         <v>1</v>
       </c>
       <c r="C20" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D20" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E20" s="3" t="n">
         <v>23</v>
       </c>
     </row>
@@ -1026,6 +1180,12 @@
         <v>0</v>
       </c>
       <c r="C21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E21" s="3" t="n">
         <v>23</v>
       </c>
     </row>
@@ -1039,6 +1199,12 @@
         <v>0</v>
       </c>
       <c r="C22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E22" s="3" t="n">
         <v>23</v>
       </c>
     </row>
@@ -1052,6 +1218,12 @@
         <v>7</v>
       </c>
       <c r="C23" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="D23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E23" s="3" t="n">
         <v>30</v>
       </c>
     </row>
@@ -1065,6 +1237,12 @@
         <v>0</v>
       </c>
       <c r="C24" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D24" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E24" s="3" t="n">
         <v>30</v>
       </c>
     </row>
@@ -1078,6 +1256,12 @@
         <v>0</v>
       </c>
       <c r="C25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E25" s="3" t="n">
         <v>30</v>
       </c>
     </row>
@@ -1091,6 +1275,12 @@
         <v>2</v>
       </c>
       <c r="C26" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D26" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E26" s="3" t="n">
         <v>32</v>
       </c>
     </row>
@@ -1104,6 +1294,12 @@
         <v>0</v>
       </c>
       <c r="C27" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D27" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E27" s="3" t="n">
         <v>32</v>
       </c>
     </row>
@@ -1117,6 +1313,12 @@
         <v>1</v>
       </c>
       <c r="C28" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D28" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E28" s="3" t="n">
         <v>33</v>
       </c>
     </row>
@@ -1130,6 +1332,12 @@
         <v>0</v>
       </c>
       <c r="C29" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D29" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E29" s="3" t="n">
         <v>33</v>
       </c>
     </row>
@@ -1143,6 +1351,12 @@
         <v>1</v>
       </c>
       <c r="C30" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D30" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E30" s="3" t="n">
         <v>34</v>
       </c>
     </row>
@@ -1156,6 +1370,12 @@
         <v>2</v>
       </c>
       <c r="C31" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D31" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E31" s="3" t="n">
         <v>36</v>
       </c>
     </row>
@@ -1169,6 +1389,12 @@
         <v>3</v>
       </c>
       <c r="C32" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D32" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E32" s="3" t="n">
         <v>39</v>
       </c>
     </row>
@@ -1182,6 +1408,12 @@
         <v>6</v>
       </c>
       <c r="C33" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="D33" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E33" s="3" t="n">
         <v>45</v>
       </c>
     </row>
@@ -1195,6 +1427,12 @@
         <v>4</v>
       </c>
       <c r="C34" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D34" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E34" s="3" t="n">
         <v>49</v>
       </c>
     </row>
@@ -1208,6 +1446,12 @@
         <v>1</v>
       </c>
       <c r="C35" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D35" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E35" s="3" t="n">
         <v>50</v>
       </c>
     </row>
@@ -1221,6 +1465,12 @@
         <v>5</v>
       </c>
       <c r="C36" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D36" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="E36" s="3" t="n">
         <v>55</v>
       </c>
     </row>
@@ -1234,6 +1484,12 @@
         <v>0</v>
       </c>
       <c r="C37" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D37" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E37" s="3" t="n">
         <v>55</v>
       </c>
     </row>
@@ -1247,6 +1503,12 @@
         <v>0</v>
       </c>
       <c r="C38" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D38" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E38" s="3" t="n">
         <v>55</v>
       </c>
     </row>
@@ -1260,6 +1522,12 @@
         <v>0</v>
       </c>
       <c r="C39" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D39" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E39" s="3" t="n">
         <v>55</v>
       </c>
     </row>
@@ -1273,6 +1541,12 @@
         <v>0</v>
       </c>
       <c r="C40" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D40" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E40" s="3" t="n">
         <v>55</v>
       </c>
     </row>
@@ -1286,6 +1560,12 @@
         <v>5</v>
       </c>
       <c r="C41" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D41" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E41" s="3" t="n">
         <v>60</v>
       </c>
     </row>
@@ -1299,6 +1579,12 @@
         <v>3</v>
       </c>
       <c r="C42" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D42" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E42" s="3" t="n">
         <v>63</v>
       </c>
     </row>
@@ -1312,6 +1598,12 @@
         <v>3</v>
       </c>
       <c r="C43" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D43" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E43" s="3" t="n">
         <v>66</v>
       </c>
     </row>
@@ -1325,6 +1617,12 @@
         <v>1</v>
       </c>
       <c r="C44" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D44" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E44" s="3" t="n">
         <v>67</v>
       </c>
     </row>
@@ -1338,6 +1636,12 @@
         <v>0</v>
       </c>
       <c r="C45" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D45" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E45" s="3" t="n">
         <v>67</v>
       </c>
     </row>
@@ -1351,6 +1655,12 @@
         <v>0</v>
       </c>
       <c r="C46" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D46" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E46" s="3" t="n">
         <v>67</v>
       </c>
     </row>
@@ -1364,6 +1674,12 @@
         <v>0</v>
       </c>
       <c r="C47" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D47" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E47" s="3" t="n">
         <v>67</v>
       </c>
     </row>
@@ -1377,6 +1693,12 @@
         <v>2</v>
       </c>
       <c r="C48" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D48" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E48" s="3" t="n">
         <v>69</v>
       </c>
     </row>
@@ -1390,6 +1712,12 @@
         <v>1</v>
       </c>
       <c r="C49" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D49" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E49" s="3" t="n">
         <v>70</v>
       </c>
     </row>
@@ -1403,6 +1731,12 @@
         <v>0</v>
       </c>
       <c r="C50" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D50" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E50" s="3" t="n">
         <v>70</v>
       </c>
     </row>
@@ -1416,6 +1750,12 @@
         <v>0</v>
       </c>
       <c r="C51" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D51" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E51" s="3" t="n">
         <v>70</v>
       </c>
     </row>
@@ -1429,6 +1769,12 @@
         <v>0</v>
       </c>
       <c r="C52" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D52" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E52" s="3" t="n">
         <v>70</v>
       </c>
     </row>
@@ -1442,6 +1788,12 @@
         <v>9</v>
       </c>
       <c r="C53" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="D53" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E53" s="3" t="n">
         <v>79</v>
       </c>
     </row>
@@ -1455,6 +1807,12 @@
         <v>8</v>
       </c>
       <c r="C54" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="D54" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E54" s="3" t="n">
         <v>87</v>
       </c>
     </row>
@@ -1468,6 +1826,12 @@
         <v>1</v>
       </c>
       <c r="C55" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D55" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E55" s="3" t="n">
         <v>88</v>
       </c>
     </row>
@@ -1481,6 +1845,12 @@
         <v>0</v>
       </c>
       <c r="C56" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D56" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E56" s="3" t="n">
         <v>88</v>
       </c>
     </row>
@@ -1494,6 +1864,12 @@
         <v>1</v>
       </c>
       <c r="C57" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D57" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E57" s="3" t="n">
         <v>89</v>
       </c>
     </row>
@@ -1507,6 +1883,12 @@
         <v>0</v>
       </c>
       <c r="C58" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D58" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E58" s="3" t="n">
         <v>89</v>
       </c>
     </row>
@@ -1520,6 +1902,12 @@
         <v>1</v>
       </c>
       <c r="C59" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D59" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E59" s="3" t="n">
         <v>90</v>
       </c>
     </row>
@@ -1533,6 +1921,12 @@
         <v>9</v>
       </c>
       <c r="C60" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="D60" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="E60" s="3" t="n">
         <v>99</v>
       </c>
     </row>
@@ -1546,6 +1940,12 @@
         <v>7</v>
       </c>
       <c r="C61" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="D61" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E61" s="3" t="n">
         <v>106</v>
       </c>
     </row>
@@ -1559,6 +1959,12 @@
         <v>2</v>
       </c>
       <c r="C62" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D62" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E62" s="3" t="n">
         <v>108</v>
       </c>
     </row>
@@ -1572,6 +1978,12 @@
         <v>0</v>
       </c>
       <c r="C63" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D63" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E63" s="3" t="n">
         <v>108</v>
       </c>
     </row>
@@ -1585,6 +1997,12 @@
         <v>7</v>
       </c>
       <c r="C64" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D64" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="E64" s="3" t="n">
         <v>115</v>
       </c>
     </row>
@@ -1598,6 +2016,12 @@
         <v>0</v>
       </c>
       <c r="C65" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D65" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E65" s="3" t="n">
         <v>115</v>
       </c>
     </row>
@@ -1611,6 +2035,12 @@
         <v>2</v>
       </c>
       <c r="C66" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D66" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E66" s="3" t="n">
         <v>117</v>
       </c>
     </row>
@@ -1624,6 +2054,12 @@
         <v>3</v>
       </c>
       <c r="C67" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="D67" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E67" s="3" t="n">
         <v>120</v>
       </c>
     </row>
@@ -1637,6 +2073,12 @@
         <v>4</v>
       </c>
       <c r="C68" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D68" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E68" s="3" t="n">
         <v>124</v>
       </c>
     </row>
@@ -1650,6 +2092,12 @@
         <v>10</v>
       </c>
       <c r="C69" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D69" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="E69" s="3" t="n">
         <v>134</v>
       </c>
     </row>
@@ -1663,6 +2111,12 @@
         <v>1</v>
       </c>
       <c r="C70" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D70" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E70" s="3" t="n">
         <v>135</v>
       </c>
     </row>
@@ -1676,6 +2130,12 @@
         <v>3</v>
       </c>
       <c r="C71" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D71" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E71" s="3" t="n">
         <v>138</v>
       </c>
     </row>
@@ -1689,6 +2149,12 @@
         <v>0</v>
       </c>
       <c r="C72" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D72" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E72" s="3" t="n">
         <v>138</v>
       </c>
     </row>
@@ -1702,6 +2168,12 @@
         <v>1</v>
       </c>
       <c r="C73" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D73" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E73" s="3" t="n">
         <v>139</v>
       </c>
     </row>
@@ -1715,6 +2187,12 @@
         <v>3</v>
       </c>
       <c r="C74" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D74" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E74" s="3" t="n">
         <v>142</v>
       </c>
     </row>
@@ -1728,6 +2206,12 @@
         <v>1</v>
       </c>
       <c r="C75" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D75" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E75" s="3" t="n">
         <v>143</v>
       </c>
     </row>
@@ -1741,6 +2225,12 @@
         <v>0</v>
       </c>
       <c r="C76" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D76" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E76" s="3" t="n">
         <v>143</v>
       </c>
     </row>
@@ -1754,6 +2244,12 @@
         <v>0</v>
       </c>
       <c r="C77" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D77" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E77" s="3" t="n">
         <v>143</v>
       </c>
     </row>
@@ -1767,6 +2263,12 @@
         <v>0</v>
       </c>
       <c r="C78" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D78" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E78" s="3" t="n">
         <v>143</v>
       </c>
     </row>
@@ -1780,6 +2282,12 @@
         <v>2</v>
       </c>
       <c r="C79" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D79" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E79" s="3" t="n">
         <v>145</v>
       </c>
     </row>
@@ -1793,6 +2301,12 @@
         <v>0</v>
       </c>
       <c r="C80" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D80" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E80" s="3" t="n">
         <v>145</v>
       </c>
     </row>
@@ -1806,6 +2320,12 @@
         <v>2</v>
       </c>
       <c r="C81" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D81" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E81" s="3" t="n">
         <v>147</v>
       </c>
     </row>
@@ -1819,6 +2339,12 @@
         <v>3</v>
       </c>
       <c r="C82" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D82" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E82" s="3" t="n">
         <v>150</v>
       </c>
     </row>
@@ -1832,6 +2358,12 @@
         <v>1</v>
       </c>
       <c r="C83" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D83" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E83" s="3" t="n">
         <v>151</v>
       </c>
     </row>
@@ -1845,6 +2377,12 @@
         <v>1</v>
       </c>
       <c r="C84" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D84" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E84" s="3" t="n">
         <v>152</v>
       </c>
     </row>
@@ -1858,6 +2396,12 @@
         <v>1</v>
       </c>
       <c r="C85" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D85" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E85" s="3" t="n">
         <v>153</v>
       </c>
     </row>
@@ -1871,6 +2415,12 @@
         <v>5</v>
       </c>
       <c r="C86" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D86" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E86" s="3" t="n">
         <v>158</v>
       </c>
     </row>
@@ -1884,6 +2434,12 @@
         <v>3</v>
       </c>
       <c r="C87" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D87" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E87" s="3" t="n">
         <v>161</v>
       </c>
     </row>
@@ -1897,6 +2453,12 @@
         <v>3</v>
       </c>
       <c r="C88" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D88" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E88" s="3" t="n">
         <v>164</v>
       </c>
     </row>
@@ -1910,6 +2472,12 @@
         <v>2</v>
       </c>
       <c r="C89" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D89" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E89" s="3" t="n">
         <v>166</v>
       </c>
     </row>
@@ -1923,6 +2491,12 @@
         <v>0</v>
       </c>
       <c r="C90" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D90" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E90" s="3" t="n">
         <v>166</v>
       </c>
     </row>
@@ -1936,6 +2510,12 @@
         <v>2</v>
       </c>
       <c r="C91" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D91" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E91" s="3" t="n">
         <v>168</v>
       </c>
     </row>
@@ -1949,6 +2529,12 @@
         <v>13</v>
       </c>
       <c r="C92" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="D92" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="E92" s="3" t="n">
         <v>181</v>
       </c>
     </row>
@@ -1962,6 +2548,12 @@
         <v>15</v>
       </c>
       <c r="C93" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="D93" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="E93" s="3" t="n">
         <v>196</v>
       </c>
     </row>
@@ -1975,6 +2567,12 @@
         <v>15</v>
       </c>
       <c r="C94" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="D94" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E94" s="3" t="n">
         <v>211</v>
       </c>
     </row>
@@ -1988,6 +2586,12 @@
         <v>20</v>
       </c>
       <c r="C95" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="D95" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E95" s="3" t="n">
         <v>231</v>
       </c>
     </row>
@@ -2001,6 +2605,12 @@
         <v>12</v>
       </c>
       <c r="C96" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="D96" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E96" s="3" t="n">
         <v>243</v>
       </c>
     </row>
@@ -2014,6 +2624,12 @@
         <v>11</v>
       </c>
       <c r="C97" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="D97" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E97" s="3" t="n">
         <v>254</v>
       </c>
     </row>
@@ -2027,6 +2643,12 @@
         <v>11</v>
       </c>
       <c r="C98" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="D98" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E98" s="3" t="n">
         <v>265</v>
       </c>
     </row>
@@ -2040,6 +2662,12 @@
         <v>3</v>
       </c>
       <c r="C99" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="D99" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E99" s="3" t="n">
         <v>268</v>
       </c>
     </row>
@@ -2053,6 +2681,12 @@
         <v>3</v>
       </c>
       <c r="C100" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D100" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E100" s="3" t="n">
         <v>271</v>
       </c>
     </row>
@@ -2066,6 +2700,12 @@
         <v>4</v>
       </c>
       <c r="C101" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="D101" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E101" s="3" t="n">
         <v>275</v>
       </c>
     </row>
@@ -2079,6 +2719,12 @@
         <v>8</v>
       </c>
       <c r="C102" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="D102" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E102" s="3" t="n">
         <v>283</v>
       </c>
     </row>
@@ -2092,6 +2738,12 @@
         <v>4</v>
       </c>
       <c r="C103" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="D103" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E103" s="3" t="n">
         <v>287</v>
       </c>
     </row>
@@ -2105,6 +2757,12 @@
         <v>8</v>
       </c>
       <c r="C104" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="D104" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E104" s="3" t="n">
         <v>295</v>
       </c>
     </row>
@@ -2118,6 +2776,12 @@
         <v>6</v>
       </c>
       <c r="C105" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="D105" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E105" s="3" t="n">
         <v>301</v>
       </c>
     </row>
@@ -2131,6 +2795,12 @@
         <v>6</v>
       </c>
       <c r="C106" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="D106" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E106" s="3" t="n">
         <v>307</v>
       </c>
     </row>
@@ -2144,6 +2814,12 @@
         <v>19</v>
       </c>
       <c r="C107" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="D107" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E107" s="3" t="n">
         <v>326</v>
       </c>
     </row>
@@ -2157,6 +2833,12 @@
         <v>8</v>
       </c>
       <c r="C108" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="D108" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E108" s="3" t="n">
         <v>334</v>
       </c>
     </row>
@@ -2172,14 +2854,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2195,15 +2878,20 @@
       </c>
       <c r="C1" s="4" t="inlineStr">
         <is>
+          <t>εκ των οποίων via Yutori</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
           <t>Ημέρες με links</t>
         </is>
       </c>
-      <c r="D1" s="4" t="inlineStr">
+      <c r="E1" s="4" t="inlineStr">
         <is>
           <t>Μέγιστο ημέρας</t>
         </is>
       </c>
-      <c r="E1" s="4" t="inlineStr">
+      <c r="F1" s="4" t="inlineStr">
         <is>
           <t>Ημερομηνία μεγίστου</t>
         </is>
@@ -2219,12 +2907,15 @@
         <v>34</v>
       </c>
       <c r="C2" s="3" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="D2" s="3" t="n">
         <v>10</v>
       </c>
-      <c r="E2" s="3" t="inlineStr">
+      <c r="E2" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
         <is>
           <t>01/05</t>
         </is>
@@ -2240,12 +2931,15 @@
         <v>63</v>
       </c>
       <c r="C3" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="D3" s="3" t="n">
         <v>17</v>
       </c>
-      <c r="D3" s="3" t="n">
+      <c r="E3" s="3" t="n">
         <v>9</v>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="F3" s="3" t="inlineStr">
         <is>
           <t>27/06</t>
         </is>
@@ -2261,12 +2955,15 @@
         <v>103</v>
       </c>
       <c r="C4" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="D4" s="3" t="n">
         <v>24</v>
       </c>
-      <c r="D4" s="3" t="n">
+      <c r="E4" s="3" t="n">
         <v>15</v>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="F4" s="3" t="inlineStr">
         <is>
           <t>31/07</t>
         </is>
@@ -2282,12 +2979,15 @@
         <v>123</v>
       </c>
       <c r="C5" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="D5" s="3" t="n">
         <v>14</v>
       </c>
-      <c r="D5" s="3" t="n">
+      <c r="E5" s="3" t="n">
         <v>20</v>
       </c>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="F5" s="3" t="inlineStr">
         <is>
           <t>01/08</t>
         </is>
@@ -2302,17 +3002,20 @@
       <c r="B6" s="3" t="n">
         <v>11</v>
       </c>
-      <c r="C6" s="3" t="inlineStr">
+      <c r="C6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D6" s="3" t="inlineStr">
+      <c r="E6" s="3" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E6" s="3" t="inlineStr">
+      <c r="F6" s="3" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2327,17 +3030,20 @@
       <c r="B7" s="5" t="n">
         <v>334</v>
       </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="C7" s="5" t="n">
+        <v>101</v>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
+      <c r="E7" s="3" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E7" s="3" t="inlineStr">
+      <c r="F7" s="3" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
Revert per-source columns in progress xlsx
Το xlsx επιστρέφει στην απλή μορφή [Ημερομηνία | Νέα Links ημέρας |
Σύνολο Links] με ένα γράφημα ημερήσιας κατανομής και ένα σωρευτικό.
Η προέλευση κάθε συνδέσμου δεν χρειάζεται στο xlsx· οι σύνδεσμοι από τα
Yutori emails εξακολουθούν να περνούν κανονικά στη συλλογή, με την ένδειξη
«(via Yutori Scout)» στο LINKS, και μετρώνται στα σύνολα.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ΠΡΟΟΔΟΣ_ΣΥΛΛΟΓΗΣ_2026.xlsx
+++ b/ΠΡΟΟΔΟΣ_ΣΥΛΛΟΓΗΣ_2026.xlsx
@@ -186,7 +186,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Νέα links ανά ημέρα ανά πηγή — Δασικές Πυρκαγιές Ελλάδα 2026</a:t>
+              <a:t>Νέα links ανά ημέρα — Δασικές Πυρκαγιές Ελλάδα 2026</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -195,13 +195,13 @@
     <plotArea>
       <barChart>
         <barDir val="col"/>
-        <grouping val="stacked"/>
+        <grouping val="clustered"/>
         <ser>
           <idx val="0"/>
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Ημερήσια Πρόοδος'!C1</f>
+              <f>'Ημερήσια Πρόοδος'!B1</f>
             </strRef>
           </tx>
           <spPr>
@@ -216,36 +216,11 @@
           </cat>
           <val>
             <numRef>
-              <f>'Ημερήσια Πρόοδος'!$C$2:$C$108</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="1"/>
-          <order val="1"/>
-          <tx>
-            <strRef>
-              <f>'Ημερήσια Πρόοδος'!D1</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'Ημερήσια Πρόοδος'!$A$3:$A$108</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Ημερήσια Πρόοδος'!$D$2:$D$108</f>
+              <f>'Ημερήσια Πρόοδος'!$B$2:$B$108</f>
             </numRef>
           </val>
         </ser>
         <gapWidth val="40"/>
-        <overlap val="100"/>
         <axId val="10"/>
         <axId val="100"/>
       </barChart>
@@ -306,9 +281,6 @@
         <crossAx val="10"/>
       </valAx>
     </plotArea>
-    <legend>
-      <legendPos val="r"/>
-    </legend>
     <plotVisOnly val="1"/>
     <dispBlanksAs val="gap"/>
   </chart>
@@ -341,7 +313,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Ημερήσια Πρόοδος'!E1</f>
+              <f>'Ημερήσια Πρόοδος'!C1</f>
             </strRef>
           </tx>
           <spPr>
@@ -364,7 +336,7 @@
           </cat>
           <val>
             <numRef>
-              <f>'Ημερήσια Πρόοδος'!$E$2:$E$108</f>
+              <f>'Ημερήσια Πρόοδος'!$C$2:$C$108</f>
             </numRef>
           </val>
         </ser>
@@ -438,7 +410,7 @@
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
-      <col>6</col>
+      <col>4</col>
       <colOff>0</colOff>
       <row>1</row>
       <rowOff>0</rowOff>
@@ -460,7 +432,7 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>6</col>
+      <col>4</col>
       <colOff>0</colOff>
       <row>21</row>
       <rowOff>0</rowOff>
@@ -772,14 +744,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E108"/>
+  <dimension ref="A1:C108"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -795,16 +765,6 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Λοιπές πηγές (web)</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>via Yutori Scout</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
           <t>Σύνολο Links</t>
         </is>
       </c>
@@ -821,12 +781,6 @@
       <c r="C2" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="D2" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E2" s="2" t="n">
-        <v>11</v>
-      </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -838,12 +792,6 @@
         <v>10</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>10</v>
-      </c>
-      <c r="D3" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E3" s="3" t="n">
         <v>21</v>
       </c>
     </row>
@@ -857,12 +805,6 @@
         <v>1</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D4" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E4" s="3" t="n">
         <v>22</v>
       </c>
     </row>
@@ -876,12 +818,6 @@
         <v>0</v>
       </c>
       <c r="C5" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D5" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E5" s="3" t="n">
         <v>22</v>
       </c>
     </row>
@@ -895,12 +831,6 @@
         <v>0</v>
       </c>
       <c r="C6" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D6" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E6" s="3" t="n">
         <v>22</v>
       </c>
     </row>
@@ -914,12 +844,6 @@
         <v>0</v>
       </c>
       <c r="C7" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D7" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E7" s="3" t="n">
         <v>22</v>
       </c>
     </row>
@@ -933,12 +857,6 @@
         <v>0</v>
       </c>
       <c r="C8" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D8" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E8" s="3" t="n">
         <v>22</v>
       </c>
     </row>
@@ -952,12 +870,6 @@
         <v>0</v>
       </c>
       <c r="C9" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D9" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E9" s="3" t="n">
         <v>22</v>
       </c>
     </row>
@@ -971,12 +883,6 @@
         <v>0</v>
       </c>
       <c r="C10" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D10" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E10" s="3" t="n">
         <v>22</v>
       </c>
     </row>
@@ -990,12 +896,6 @@
         <v>0</v>
       </c>
       <c r="C11" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D11" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E11" s="3" t="n">
         <v>22</v>
       </c>
     </row>
@@ -1009,12 +909,6 @@
         <v>0</v>
       </c>
       <c r="C12" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D12" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E12" s="3" t="n">
         <v>22</v>
       </c>
     </row>
@@ -1028,12 +922,6 @@
         <v>0</v>
       </c>
       <c r="C13" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D13" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E13" s="3" t="n">
         <v>22</v>
       </c>
     </row>
@@ -1047,12 +935,6 @@
         <v>0</v>
       </c>
       <c r="C14" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D14" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E14" s="3" t="n">
         <v>22</v>
       </c>
     </row>
@@ -1066,12 +948,6 @@
         <v>0</v>
       </c>
       <c r="C15" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D15" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E15" s="3" t="n">
         <v>22</v>
       </c>
     </row>
@@ -1085,12 +961,6 @@
         <v>0</v>
       </c>
       <c r="C16" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D16" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E16" s="3" t="n">
         <v>22</v>
       </c>
     </row>
@@ -1104,12 +974,6 @@
         <v>0</v>
       </c>
       <c r="C17" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D17" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E17" s="3" t="n">
         <v>22</v>
       </c>
     </row>
@@ -1123,12 +987,6 @@
         <v>0</v>
       </c>
       <c r="C18" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D18" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E18" s="3" t="n">
         <v>22</v>
       </c>
     </row>
@@ -1142,12 +1000,6 @@
         <v>0</v>
       </c>
       <c r="C19" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D19" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E19" s="3" t="n">
         <v>22</v>
       </c>
     </row>
@@ -1161,12 +1013,6 @@
         <v>1</v>
       </c>
       <c r="C20" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D20" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E20" s="3" t="n">
         <v>23</v>
       </c>
     </row>
@@ -1180,12 +1026,6 @@
         <v>0</v>
       </c>
       <c r="C21" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D21" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E21" s="3" t="n">
         <v>23</v>
       </c>
     </row>
@@ -1199,12 +1039,6 @@
         <v>0</v>
       </c>
       <c r="C22" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D22" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E22" s="3" t="n">
         <v>23</v>
       </c>
     </row>
@@ -1218,12 +1052,6 @@
         <v>7</v>
       </c>
       <c r="C23" s="3" t="n">
-        <v>7</v>
-      </c>
-      <c r="D23" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E23" s="3" t="n">
         <v>30</v>
       </c>
     </row>
@@ -1237,12 +1065,6 @@
         <v>0</v>
       </c>
       <c r="C24" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D24" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E24" s="3" t="n">
         <v>30</v>
       </c>
     </row>
@@ -1256,12 +1078,6 @@
         <v>0</v>
       </c>
       <c r="C25" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D25" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E25" s="3" t="n">
         <v>30</v>
       </c>
     </row>
@@ -1275,12 +1091,6 @@
         <v>2</v>
       </c>
       <c r="C26" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="D26" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E26" s="3" t="n">
         <v>32</v>
       </c>
     </row>
@@ -1294,12 +1104,6 @@
         <v>0</v>
       </c>
       <c r="C27" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D27" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E27" s="3" t="n">
         <v>32</v>
       </c>
     </row>
@@ -1313,12 +1117,6 @@
         <v>1</v>
       </c>
       <c r="C28" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D28" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E28" s="3" t="n">
         <v>33</v>
       </c>
     </row>
@@ -1332,12 +1130,6 @@
         <v>0</v>
       </c>
       <c r="C29" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D29" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E29" s="3" t="n">
         <v>33</v>
       </c>
     </row>
@@ -1351,12 +1143,6 @@
         <v>1</v>
       </c>
       <c r="C30" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D30" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E30" s="3" t="n">
         <v>34</v>
       </c>
     </row>
@@ -1370,12 +1156,6 @@
         <v>2</v>
       </c>
       <c r="C31" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="D31" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E31" s="3" t="n">
         <v>36</v>
       </c>
     </row>
@@ -1389,12 +1169,6 @@
         <v>3</v>
       </c>
       <c r="C32" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D32" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="E32" s="3" t="n">
         <v>39</v>
       </c>
     </row>
@@ -1408,12 +1182,6 @@
         <v>6</v>
       </c>
       <c r="C33" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="D33" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="E33" s="3" t="n">
         <v>45</v>
       </c>
     </row>
@@ -1427,12 +1195,6 @@
         <v>4</v>
       </c>
       <c r="C34" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="D34" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="E34" s="3" t="n">
         <v>49</v>
       </c>
     </row>
@@ -1446,12 +1208,6 @@
         <v>1</v>
       </c>
       <c r="C35" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D35" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E35" s="3" t="n">
         <v>50</v>
       </c>
     </row>
@@ -1465,12 +1221,6 @@
         <v>5</v>
       </c>
       <c r="C36" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D36" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="E36" s="3" t="n">
         <v>55</v>
       </c>
     </row>
@@ -1484,12 +1234,6 @@
         <v>0</v>
       </c>
       <c r="C37" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D37" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E37" s="3" t="n">
         <v>55</v>
       </c>
     </row>
@@ -1503,12 +1247,6 @@
         <v>0</v>
       </c>
       <c r="C38" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D38" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E38" s="3" t="n">
         <v>55</v>
       </c>
     </row>
@@ -1522,12 +1260,6 @@
         <v>0</v>
       </c>
       <c r="C39" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D39" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E39" s="3" t="n">
         <v>55</v>
       </c>
     </row>
@@ -1541,12 +1273,6 @@
         <v>0</v>
       </c>
       <c r="C40" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D40" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E40" s="3" t="n">
         <v>55</v>
       </c>
     </row>
@@ -1560,12 +1286,6 @@
         <v>5</v>
       </c>
       <c r="C41" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="D41" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="E41" s="3" t="n">
         <v>60</v>
       </c>
     </row>
@@ -1579,12 +1299,6 @@
         <v>3</v>
       </c>
       <c r="C42" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D42" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="E42" s="3" t="n">
         <v>63</v>
       </c>
     </row>
@@ -1598,12 +1312,6 @@
         <v>3</v>
       </c>
       <c r="C43" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D43" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="E43" s="3" t="n">
         <v>66</v>
       </c>
     </row>
@@ -1617,12 +1325,6 @@
         <v>1</v>
       </c>
       <c r="C44" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D44" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E44" s="3" t="n">
         <v>67</v>
       </c>
     </row>
@@ -1636,12 +1338,6 @@
         <v>0</v>
       </c>
       <c r="C45" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D45" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E45" s="3" t="n">
         <v>67</v>
       </c>
     </row>
@@ -1655,12 +1351,6 @@
         <v>0</v>
       </c>
       <c r="C46" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D46" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E46" s="3" t="n">
         <v>67</v>
       </c>
     </row>
@@ -1674,12 +1364,6 @@
         <v>0</v>
       </c>
       <c r="C47" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D47" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E47" s="3" t="n">
         <v>67</v>
       </c>
     </row>
@@ -1693,12 +1377,6 @@
         <v>2</v>
       </c>
       <c r="C48" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="D48" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E48" s="3" t="n">
         <v>69</v>
       </c>
     </row>
@@ -1712,12 +1390,6 @@
         <v>1</v>
       </c>
       <c r="C49" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D49" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E49" s="3" t="n">
         <v>70</v>
       </c>
     </row>
@@ -1731,12 +1403,6 @@
         <v>0</v>
       </c>
       <c r="C50" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D50" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E50" s="3" t="n">
         <v>70</v>
       </c>
     </row>
@@ -1750,12 +1416,6 @@
         <v>0</v>
       </c>
       <c r="C51" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D51" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E51" s="3" t="n">
         <v>70</v>
       </c>
     </row>
@@ -1769,12 +1429,6 @@
         <v>0</v>
       </c>
       <c r="C52" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D52" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E52" s="3" t="n">
         <v>70</v>
       </c>
     </row>
@@ -1788,12 +1442,6 @@
         <v>9</v>
       </c>
       <c r="C53" s="3" t="n">
-        <v>9</v>
-      </c>
-      <c r="D53" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E53" s="3" t="n">
         <v>79</v>
       </c>
     </row>
@@ -1807,12 +1455,6 @@
         <v>8</v>
       </c>
       <c r="C54" s="3" t="n">
-        <v>8</v>
-      </c>
-      <c r="D54" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E54" s="3" t="n">
         <v>87</v>
       </c>
     </row>
@@ -1826,12 +1468,6 @@
         <v>1</v>
       </c>
       <c r="C55" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D55" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E55" s="3" t="n">
         <v>88</v>
       </c>
     </row>
@@ -1845,12 +1481,6 @@
         <v>0</v>
       </c>
       <c r="C56" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D56" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E56" s="3" t="n">
         <v>88</v>
       </c>
     </row>
@@ -1864,12 +1494,6 @@
         <v>1</v>
       </c>
       <c r="C57" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D57" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E57" s="3" t="n">
         <v>89</v>
       </c>
     </row>
@@ -1883,12 +1507,6 @@
         <v>0</v>
       </c>
       <c r="C58" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D58" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E58" s="3" t="n">
         <v>89</v>
       </c>
     </row>
@@ -1902,12 +1520,6 @@
         <v>1</v>
       </c>
       <c r="C59" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D59" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E59" s="3" t="n">
         <v>90</v>
       </c>
     </row>
@@ -1921,12 +1533,6 @@
         <v>9</v>
       </c>
       <c r="C60" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="D60" s="3" t="n">
-        <v>6</v>
-      </c>
-      <c r="E60" s="3" t="n">
         <v>99</v>
       </c>
     </row>
@@ -1940,12 +1546,6 @@
         <v>7</v>
       </c>
       <c r="C61" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="D61" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="E61" s="3" t="n">
         <v>106</v>
       </c>
     </row>
@@ -1959,12 +1559,6 @@
         <v>2</v>
       </c>
       <c r="C62" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D62" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="E62" s="3" t="n">
         <v>108</v>
       </c>
     </row>
@@ -1978,12 +1572,6 @@
         <v>0</v>
       </c>
       <c r="C63" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D63" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E63" s="3" t="n">
         <v>108</v>
       </c>
     </row>
@@ -1997,12 +1585,6 @@
         <v>7</v>
       </c>
       <c r="C64" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D64" s="3" t="n">
-        <v>6</v>
-      </c>
-      <c r="E64" s="3" t="n">
         <v>115</v>
       </c>
     </row>
@@ -2016,12 +1598,6 @@
         <v>0</v>
       </c>
       <c r="C65" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D65" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E65" s="3" t="n">
         <v>115</v>
       </c>
     </row>
@@ -2035,12 +1611,6 @@
         <v>2</v>
       </c>
       <c r="C66" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="D66" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E66" s="3" t="n">
         <v>117</v>
       </c>
     </row>
@@ -2054,12 +1624,6 @@
         <v>3</v>
       </c>
       <c r="C67" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="D67" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E67" s="3" t="n">
         <v>120</v>
       </c>
     </row>
@@ -2073,12 +1637,6 @@
         <v>4</v>
       </c>
       <c r="C68" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="D68" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="E68" s="3" t="n">
         <v>124</v>
       </c>
     </row>
@@ -2092,12 +1650,6 @@
         <v>10</v>
       </c>
       <c r="C69" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="D69" s="3" t="n">
-        <v>8</v>
-      </c>
-      <c r="E69" s="3" t="n">
         <v>134</v>
       </c>
     </row>
@@ -2111,12 +1663,6 @@
         <v>1</v>
       </c>
       <c r="C70" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D70" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E70" s="3" t="n">
         <v>135</v>
       </c>
     </row>
@@ -2130,12 +1676,6 @@
         <v>3</v>
       </c>
       <c r="C71" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D71" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="E71" s="3" t="n">
         <v>138</v>
       </c>
     </row>
@@ -2149,12 +1689,6 @@
         <v>0</v>
       </c>
       <c r="C72" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D72" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E72" s="3" t="n">
         <v>138</v>
       </c>
     </row>
@@ -2168,12 +1702,6 @@
         <v>1</v>
       </c>
       <c r="C73" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D73" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E73" s="3" t="n">
         <v>139</v>
       </c>
     </row>
@@ -2187,12 +1715,6 @@
         <v>3</v>
       </c>
       <c r="C74" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D74" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="E74" s="3" t="n">
         <v>142</v>
       </c>
     </row>
@@ -2206,12 +1728,6 @@
         <v>1</v>
       </c>
       <c r="C75" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D75" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E75" s="3" t="n">
         <v>143</v>
       </c>
     </row>
@@ -2225,12 +1741,6 @@
         <v>0</v>
       </c>
       <c r="C76" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D76" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E76" s="3" t="n">
         <v>143</v>
       </c>
     </row>
@@ -2244,12 +1754,6 @@
         <v>0</v>
       </c>
       <c r="C77" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D77" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E77" s="3" t="n">
         <v>143</v>
       </c>
     </row>
@@ -2263,12 +1767,6 @@
         <v>0</v>
       </c>
       <c r="C78" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D78" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E78" s="3" t="n">
         <v>143</v>
       </c>
     </row>
@@ -2282,12 +1780,6 @@
         <v>2</v>
       </c>
       <c r="C79" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D79" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E79" s="3" t="n">
         <v>145</v>
       </c>
     </row>
@@ -2301,12 +1793,6 @@
         <v>0</v>
       </c>
       <c r="C80" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D80" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E80" s="3" t="n">
         <v>145</v>
       </c>
     </row>
@@ -2320,12 +1806,6 @@
         <v>2</v>
       </c>
       <c r="C81" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="D81" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E81" s="3" t="n">
         <v>147</v>
       </c>
     </row>
@@ -2339,12 +1819,6 @@
         <v>3</v>
       </c>
       <c r="C82" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D82" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="E82" s="3" t="n">
         <v>150</v>
       </c>
     </row>
@@ -2358,12 +1832,6 @@
         <v>1</v>
       </c>
       <c r="C83" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D83" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E83" s="3" t="n">
         <v>151</v>
       </c>
     </row>
@@ -2377,12 +1845,6 @@
         <v>1</v>
       </c>
       <c r="C84" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D84" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E84" s="3" t="n">
         <v>152</v>
       </c>
     </row>
@@ -2396,12 +1858,6 @@
         <v>1</v>
       </c>
       <c r="C85" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D85" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E85" s="3" t="n">
         <v>153</v>
       </c>
     </row>
@@ -2415,12 +1871,6 @@
         <v>5</v>
       </c>
       <c r="C86" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="D86" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="E86" s="3" t="n">
         <v>158</v>
       </c>
     </row>
@@ -2434,12 +1884,6 @@
         <v>3</v>
       </c>
       <c r="C87" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="D87" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E87" s="3" t="n">
         <v>161</v>
       </c>
     </row>
@@ -2453,12 +1897,6 @@
         <v>3</v>
       </c>
       <c r="C88" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D88" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="E88" s="3" t="n">
         <v>164</v>
       </c>
     </row>
@@ -2472,12 +1910,6 @@
         <v>2</v>
       </c>
       <c r="C89" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D89" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E89" s="3" t="n">
         <v>166</v>
       </c>
     </row>
@@ -2491,12 +1923,6 @@
         <v>0</v>
       </c>
       <c r="C90" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D90" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E90" s="3" t="n">
         <v>166</v>
       </c>
     </row>
@@ -2510,12 +1936,6 @@
         <v>2</v>
       </c>
       <c r="C91" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D91" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E91" s="3" t="n">
         <v>168</v>
       </c>
     </row>
@@ -2529,12 +1949,6 @@
         <v>13</v>
       </c>
       <c r="C92" s="3" t="n">
-        <v>8</v>
-      </c>
-      <c r="D92" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="E92" s="3" t="n">
         <v>181</v>
       </c>
     </row>
@@ -2548,12 +1962,6 @@
         <v>15</v>
       </c>
       <c r="C93" s="3" t="n">
-        <v>10</v>
-      </c>
-      <c r="D93" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="E93" s="3" t="n">
         <v>196</v>
       </c>
     </row>
@@ -2567,12 +1975,6 @@
         <v>15</v>
       </c>
       <c r="C94" s="3" t="n">
-        <v>13</v>
-      </c>
-      <c r="D94" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="E94" s="3" t="n">
         <v>211</v>
       </c>
     </row>
@@ -2586,12 +1988,6 @@
         <v>20</v>
       </c>
       <c r="C95" s="3" t="n">
-        <v>19</v>
-      </c>
-      <c r="D95" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E95" s="3" t="n">
         <v>231</v>
       </c>
     </row>
@@ -2605,12 +2001,6 @@
         <v>12</v>
       </c>
       <c r="C96" s="3" t="n">
-        <v>10</v>
-      </c>
-      <c r="D96" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="E96" s="3" t="n">
         <v>243</v>
       </c>
     </row>
@@ -2624,12 +2014,6 @@
         <v>11</v>
       </c>
       <c r="C97" s="3" t="n">
-        <v>8</v>
-      </c>
-      <c r="D97" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="E97" s="3" t="n">
         <v>254</v>
       </c>
     </row>
@@ -2643,12 +2027,6 @@
         <v>11</v>
       </c>
       <c r="C98" s="3" t="n">
-        <v>9</v>
-      </c>
-      <c r="D98" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="E98" s="3" t="n">
         <v>265</v>
       </c>
     </row>
@@ -2662,12 +2040,6 @@
         <v>3</v>
       </c>
       <c r="C99" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="D99" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E99" s="3" t="n">
         <v>268</v>
       </c>
     </row>
@@ -2681,12 +2053,6 @@
         <v>3</v>
       </c>
       <c r="C100" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="D100" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E100" s="3" t="n">
         <v>271</v>
       </c>
     </row>
@@ -2700,12 +2066,6 @@
         <v>4</v>
       </c>
       <c r="C101" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="D101" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E101" s="3" t="n">
         <v>275</v>
       </c>
     </row>
@@ -2719,12 +2079,6 @@
         <v>8</v>
       </c>
       <c r="C102" s="3" t="n">
-        <v>6</v>
-      </c>
-      <c r="D102" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="E102" s="3" t="n">
         <v>283</v>
       </c>
     </row>
@@ -2738,12 +2092,6 @@
         <v>4</v>
       </c>
       <c r="C103" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="D103" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E103" s="3" t="n">
         <v>287</v>
       </c>
     </row>
@@ -2757,12 +2105,6 @@
         <v>8</v>
       </c>
       <c r="C104" s="3" t="n">
-        <v>7</v>
-      </c>
-      <c r="D104" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E104" s="3" t="n">
         <v>295</v>
       </c>
     </row>
@@ -2776,12 +2118,6 @@
         <v>6</v>
       </c>
       <c r="C105" s="3" t="n">
-        <v>6</v>
-      </c>
-      <c r="D105" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E105" s="3" t="n">
         <v>301</v>
       </c>
     </row>
@@ -2795,12 +2131,6 @@
         <v>6</v>
       </c>
       <c r="C106" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="D106" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E106" s="3" t="n">
         <v>307</v>
       </c>
     </row>
@@ -2814,12 +2144,6 @@
         <v>19</v>
       </c>
       <c r="C107" s="3" t="n">
-        <v>17</v>
-      </c>
-      <c r="D107" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="E107" s="3" t="n">
         <v>326</v>
       </c>
     </row>
@@ -2833,12 +2157,6 @@
         <v>8</v>
       </c>
       <c r="C108" s="3" t="n">
-        <v>7</v>
-      </c>
-      <c r="D108" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E108" s="3" t="n">
         <v>334</v>
       </c>
     </row>
@@ -2854,15 +2172,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2878,20 +2195,15 @@
       </c>
       <c r="C1" s="4" t="inlineStr">
         <is>
-          <t>εκ των οποίων via Yutori</t>
+          <t>Ημέρες με links</t>
         </is>
       </c>
       <c r="D1" s="4" t="inlineStr">
         <is>
-          <t>Ημέρες με links</t>
+          <t>Μέγιστο ημέρας</t>
         </is>
       </c>
       <c r="E1" s="4" t="inlineStr">
-        <is>
-          <t>Μέγιστο ημέρας</t>
-        </is>
-      </c>
-      <c r="F1" s="4" t="inlineStr">
         <is>
           <t>Ημερομηνία μεγίστου</t>
         </is>
@@ -2907,15 +2219,12 @@
         <v>34</v>
       </c>
       <c r="C2" s="3" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="D2" s="3" t="n">
         <v>10</v>
       </c>
-      <c r="E2" s="3" t="n">
-        <v>10</v>
-      </c>
-      <c r="F2" s="3" t="inlineStr">
+      <c r="E2" s="3" t="inlineStr">
         <is>
           <t>01/05</t>
         </is>
@@ -2931,15 +2240,12 @@
         <v>63</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>28</v>
+        <v>17</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>17</v>
-      </c>
-      <c r="E3" s="3" t="n">
         <v>9</v>
       </c>
-      <c r="F3" s="3" t="inlineStr">
+      <c r="E3" s="3" t="inlineStr">
         <is>
           <t>27/06</t>
         </is>
@@ -2955,15 +2261,12 @@
         <v>103</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>50</v>
+        <v>24</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>24</v>
-      </c>
-      <c r="E4" s="3" t="n">
         <v>15</v>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="E4" s="3" t="inlineStr">
         <is>
           <t>31/07</t>
         </is>
@@ -2979,15 +2282,12 @@
         <v>123</v>
       </c>
       <c r="C5" s="3" t="n">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>14</v>
-      </c>
-      <c r="E5" s="3" t="n">
         <v>20</v>
       </c>
-      <c r="F5" s="3" t="inlineStr">
+      <c r="E5" s="3" t="inlineStr">
         <is>
           <t>01/08</t>
         </is>
@@ -3002,8 +2302,10 @@
       <c r="B6" s="3" t="n">
         <v>11</v>
       </c>
-      <c r="C6" s="3" t="n">
-        <v>0</v>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
@@ -3011,11 +2313,6 @@
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F6" s="3" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -3030,8 +2327,10 @@
       <c r="B7" s="5" t="n">
         <v>334</v>
       </c>
-      <c r="C7" s="5" t="n">
-        <v>101</v>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
@@ -3039,11 +2338,6 @@
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F7" s="3" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
Yutori Scout check 15/08: 0 new links, registry #8 enriched
Έλεγχος 5 αναφορών Scout (10–14/8) μέσω Gmail. Εξήχθησαν 9 URLs πηγών από
τις παραμέτρους url= των scouts.yutori.com/api/view links:
- 7 ελληνικοί σύνδεσμοι υπήρχαν ήδη στο LINKS (καμία προσθήκη)
- 2 απορρίφθηκαν ως μη ελληνικά περιστατικά (Mizerieux Γαλλίας μέσω CNN,
  Mount Barone Ιταλίας μέσω RTE)· και τα δύο domains είναι αποκλεισμένα από
  τον proxy, οπότε δεν ήταν δυνατή η επαλήθευση ελληνικού περιεχομένου

Μητρώο #8 (Σίβηρη/Φούρκα Χαλκιδικής): διάρκεια 13→14/8, δυνάμεις 14/8
(140+ πυροσβέστες, 9 αεροσκάφη, 7 ελικόπτερα), ~300+ τουρίστες εκκενωμένοι
δια θαλάσσης, προειδοποίηση Κατηγορίας 5 από 12/8, ένταξη σε έξαρση 40+
πυρκαγιών πανελλαδικά, +3 πηγές.

Σύνολο συνδέσμων αμετάβλητο: 334.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ΠΡΟΟΔΟΣ_ΣΥΛΛΟΓΗΣ_2026.xlsx
+++ b/ΠΡΟΟΔΟΣ_ΣΥΛΛΟΓΗΣ_2026.xlsx
@@ -211,12 +211,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Ημερήσια Πρόοδος'!$A$3:$A$108</f>
+              <f>'Ημερήσια Πρόοδος'!$A$3:$A$109</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Ημερήσια Πρόοδος'!$B$2:$B$108</f>
+              <f>'Ημερήσια Πρόοδος'!$B$2:$B$109</f>
             </numRef>
           </val>
         </ser>
@@ -331,12 +331,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Ημερήσια Πρόοδος'!$A$3:$A$108</f>
+              <f>'Ημερήσια Πρόοδος'!$A$3:$A$109</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Ημερήσια Πρόοδος'!$C$2:$C$108</f>
+              <f>'Ημερήσια Πρόοδος'!$C$2:$C$109</f>
             </numRef>
           </val>
         </ser>
@@ -744,7 +744,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C108"/>
+  <dimension ref="A1:C109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2157,6 +2157,19 @@
         <v>8</v>
       </c>
       <c r="C108" s="3" t="n">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="3" t="inlineStr">
+        <is>
+          <t>15/08</t>
+        </is>
+      </c>
+      <c r="B109" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C109" s="3" t="n">
         <v>334</v>
       </c>
     </row>

</xml_diff>